<commit_message>
Corrected title & semester
</commit_message>
<xml_diff>
--- a/_data/sessions.xlsx
+++ b/_data/sessions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Github/jirelations/25rw/_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0BEE00-AAB3-2241-97AC-C7ECDA762E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995AF400-B8BE-2A4E-A11C-999D816B2525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -872,7 +872,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="3">
         <v>1</v>
       </c>
@@ -958,7 +958,8 @@
 </v>
       </c>
       <c r="T2" s="15" t="str">
-        <f>"# Einführung in die Religionswissenschaft
+        <f>"# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### "&amp;G2&amp;"
 Wintersemester 2025/2026
@@ -970,7 +971,8 @@
 ## Einleitung
 ## Heutiges Lernziel
 "&amp;N2</f>
-        <v># Einführung in die Religionswissenschaft
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was machen wir hier?
 Wintersemester 2025/2026
@@ -1007,7 +1009,8 @@
 image: candle.jpg
 parallaxBackgroundImage: 'assets/img/candle.jpg'
 ---
-# Einführung in die Religionswissenschaft
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was machen wir hier?
 Wintersemester 2025/2026
@@ -1025,7 +1028,7 @@
 Was ist die Religionswissenschaft?</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3">
         <v>2</v>
       </c>
@@ -1116,10 +1119,11 @@
 </v>
       </c>
       <c r="T3" s="15" t="str">
-        <f t="shared" ref="T3:T16" si="9">"# Einführung ins Judentum
+        <f t="shared" ref="T3:T16" si="9">"# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### "&amp;G3&amp;"
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 "&amp;N2&amp;"
@@ -1128,10 +1132,11 @@
 ## Einleitung
 ## Heutiges Lernziel
 "&amp;N3</f>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was ist die Religionswissenschaft?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Sich gegenseitig kennenlernen und unsere gegenseitige Ziele für den Kurs berücksichtigen.
@@ -1165,10 +1170,11 @@
 image: religionen-lupe.jpg
 parallaxBackgroundImage: 'assets/img/religionen-lupe.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was ist die Religionswissenschaft?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Sich gegenseitig kennenlernen und unsere gegenseitige Ziele für den Kurs berücksichtigen.
@@ -1183,7 +1189,7 @@
 Was ist Religion?</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="3">
         <v>3</v>
       </c>
@@ -1260,10 +1266,11 @@
       </c>
       <c r="T4" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was ist Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Die Bestimmung des Fachs Religionswissenschaft in seiner Breite und mit seinen Unterschieden zur Theologie erfassen.
@@ -1293,10 +1300,11 @@
 image: magnifying-glass.jpg
 parallaxBackgroundImage: 'assets/img/magnifying-glass.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was ist Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Die Bestimmung des Fachs Religionswissenschaft in seiner Breite und mit seinen Unterschieden zur Theologie erfassen.
@@ -1311,7 +1319,7 @@
 Was gilt als religiöses Ritual?</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
         <v>4</v>
       </c>
@@ -1388,10 +1396,11 @@
       </c>
       <c r="T5" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was gilt als religiöses Ritual?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Verschiedene Definitionen von Religion unterscheiden können, was sie umfassen und wofür sie nützlich sein können.
@@ -1421,10 +1430,11 @@
 image: 02_Fussball.jpg
 parallaxBackgroundImage: 'assets/img/02_Fussball.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Was gilt als religiöses Ritual?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Verschiedene Definitionen von Religion unterscheiden können, was sie umfassen und wofür sie nützlich sein können.
@@ -1439,7 +1449,7 @@
 Wie bilden sich religiöse Gruppen und Autoritäten?</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
         <v>5</v>
       </c>
@@ -1513,10 +1523,11 @@
       </c>
       <c r="T6" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie bilden sich religiöse Gruppen und Autoritäten?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Rituale auf drei Ebenen (Formen, Funktionen, Bedeutungen) anhand von Beispielen schildern können.
@@ -1546,10 +1557,11 @@
 image: kaaba.jpg
 parallaxBackgroundImage: 'assets/img/kaaba.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie bilden sich religiöse Gruppen und Autoritäten?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Rituale auf drei Ebenen (Formen, Funktionen, Bedeutungen) anhand von Beispielen schildern können.
@@ -1564,7 +1576,7 @@
 Welche Rolle spielt Gender in der Religion?</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3">
         <v>6</v>
       </c>
@@ -1638,10 +1650,11 @@
       </c>
       <c r="T7" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Rolle spielt Gender in der Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Historische und gegenwärtige Beispiele der Gruppenbildung anhand eines differenzierten Konzepts von "Meister/Jüngerschaft" erläutern können.
@@ -1671,10 +1684,11 @@
 image: 04.MarabouWomen.jpg
 parallaxBackgroundImage: 'assets/img/04.MarabouWomen.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Rolle spielt Gender in der Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Historische und gegenwärtige Beispiele der Gruppenbildung anhand eines differenzierten Konzepts von "Meister/Jüngerschaft" erläutern können.
@@ -1689,7 +1703,7 @@
 Wer oder was bestimmt die Orthodoxie?</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3">
         <v>7</v>
       </c>
@@ -1763,10 +1777,11 @@
       </c>
       <c r="T8" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wer oder was bestimmt die Orthodoxie?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Ebenen der Genderforschung erläutern können, auf die die Religionswissenschaft grundlegend eingehen kann.
@@ -1796,10 +1811,11 @@
 image: yezidi.jpg
 parallaxBackgroundImage: 'assets/img/yezidi.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wer oder was bestimmt die Orthodoxie?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Ebenen der Genderforschung erläutern können, auf die die Religionswissenschaft grundlegend eingehen kann.
@@ -1814,7 +1830,7 @@
 Wie werden heilige Schriften überliefert?</v>
       </c>
     </row>
-    <row r="9" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="3">
         <v>8</v>
       </c>
@@ -1888,10 +1904,11 @@
       </c>
       <c r="T9" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie werden heilige Schriften überliefert?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Erklären können, wie Normativitätsansprüche in der Religionswissenschaft untersucht werden können.
@@ -1921,10 +1938,11 @@
 image: synagogue-scroll.jpg
 parallaxBackgroundImage: 'assets/img/synagogue-scroll.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie werden heilige Schriften überliefert?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Erklären können, wie Normativitätsansprüche in der Religionswissenschaft untersucht werden können.
@@ -1939,7 +1957,7 @@
 Welche Rolle spielen materielle Objekte in der Religion?</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3">
         <v>9</v>
       </c>
@@ -2013,10 +2031,11 @@
       </c>
       <c r="T10" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Rolle spielen materielle Objekte in der Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Die mündliche und schriftliche Dynamik der abrahamitischen Religionen im Verhältnis zueinander zu beschreiben.
@@ -2046,10 +2065,11 @@
 image: mosque.jpg
 parallaxBackgroundImage: 'assets/img/mosque.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Rolle spielen materielle Objekte in der Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Die mündliche und schriftliche Dynamik der abrahamitischen Religionen im Verhältnis zueinander zu beschreiben.
@@ -2064,7 +2084,7 @@
 Welche Rolle spielen heilige Orte in der Religion?</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3">
         <v>10</v>
       </c>
@@ -2141,10 +2161,11 @@
       </c>
       <c r="T11" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Rolle spielen heilige Orte in der Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Erklären können, wie die Forschung an materiellen Objekten den Glauben an das Transzendente greifbar macht.
@@ -2174,10 +2195,11 @@
 image: madaba-map.jpg
 parallaxBackgroundImage: 'assets/img/madaba-map.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Rolle spielen heilige Orte in der Religion?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Erklären können, wie die Forschung an materiellen Objekten den Glauben an das Transzendente greifbar macht.
@@ -2192,7 +2214,7 @@
 Welche Wirkung hat die religiöse Praxis auf den Körper?</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3">
         <v>11</v>
       </c>
@@ -2269,10 +2291,11 @@
       </c>
       <c r="T12" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Wirkung hat die religiöse Praxis auf den Körper?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Erklären können, auf welche Weise Orte sakrale Bedeutung erlangen, und diese Bedeutung anhand jüdischer, christlicher und islamischer Beispiele erläutern.
@@ -2302,10 +2325,11 @@
 image: dhanvantari.jpg
 parallaxBackgroundImage: 'assets/img/dhanvantari.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Welche Wirkung hat die religiöse Praxis auf den Körper?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Erklären können, auf welche Weise Orte sakrale Bedeutung erlangen, und diese Bedeutung anhand jüdischer, christlicher und islamischer Beispiele erläutern.
@@ -2320,7 +2344,7 @@
 Wie wird Religion digital untersucht?</v>
       </c>
     </row>
-    <row r="13" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3">
         <v>12</v>
       </c>
@@ -2397,10 +2421,11 @@
       </c>
       <c r="T13" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie wird Religion digital untersucht?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Religionspsychologische Ansätze zur Krankheit und Heilung schildern.
@@ -2430,10 +2455,11 @@
 image: digital.jpg
 parallaxBackgroundImage: 'assets/img/digital.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie wird Religion digital untersucht?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Religionspsychologische Ansätze zur Krankheit und Heilung schildern.
@@ -2448,7 +2474,7 @@
 Wie sollte religiöser Extremismus verstanden werden?</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="5">
         <v>13</v>
       </c>
@@ -2525,10 +2551,11 @@
       </c>
       <c r="T14" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie sollte religiöser Extremismus verstanden werden?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Verständnis dafür zeigen, wie religiöse Identität, Gemeinschaft und Autorität in Online- und Offline-Umgebungen miteinander verwoben sind.
@@ -2558,10 +2585,11 @@
 image: 12_iranischeSchiiten.jpeg
 parallaxBackgroundImage: 'assets/img/12_iranischeSchiiten.jpeg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie sollte religiöser Extremismus verstanden werden?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Verständnis dafür zeigen, wie religiöse Identität, Gemeinschaft und Autorität in Online- und Offline-Umgebungen miteinander verwoben sind.
@@ -2576,7 +2604,7 @@
 Sollten Religionswissenschaftler/innen am interreligiösen Dialog mitwirken?</v>
       </c>
     </row>
-    <row r="15" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="5">
         <v>14</v>
       </c>
@@ -2650,10 +2678,11 @@
       </c>
       <c r="T15" s="15" t="str">
         <f t="shared" si="9"/>
-        <v># Einführung ins Judentum
+        <v># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Sollten Religionswissenschaftler/innen am interreligiösen Dialog mitwirken?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Fundamentalismus, Radikalisierung und Extremismus definieren und Beispiele für jeden Begriff geben.
@@ -2683,10 +2712,11 @@
 image: interreligious-conversation.png
 parallaxBackgroundImage: 'assets/img/interreligious-conversation.png'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Sollten Religionswissenschaftler/innen am interreligiösen Dialog mitwirken?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Fundamentalismus, Radikalisierung und Extremismus definieren und Beispiele für jeden Begriff geben.
@@ -2701,7 +2731,7 @@
 Wie gehe ich mit dem erworbenen Wissen um?</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="5">
         <v>15</v>
       </c>
@@ -2769,10 +2799,11 @@
       </c>
       <c r="T16" s="15" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"># Einführung ins Judentum
+        <v xml:space="preserve"># Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie gehe ich mit dem erworbenen Wissen um?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Überlegen und erklären können, inwieweit religionswissenschaftliche Ansätze zum interreligiösen Dialog beitragen können, sollen und dürfen.
@@ -2802,10 +2833,11 @@
 image: girl-bridge.jpg
 parallaxBackgroundImage: 'assets/img/girl-bridge.jpg'
 ---
-# Einführung ins Judentum
+# Einführung in die 
+### Religionswissenschaft
 {: .r-fit-text}
 ### Wie gehe ich mit dem erworbenen Wissen um?
-Sommersemester 2025
+Wintersemester 2025/2026
 Prof. Dr. Nathan Gibson
 ## 📈 Rückblick: Lernziel
 Überlegen und erklären können, inwieweit religionswissenschaftliche Ansätze zum interreligiösen Dialog beitragen können, sollen und dürfen.

</xml_diff>